<commit_message>
feat(crew): configure hyperspace time efficiency and luck
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/crew_config.xlsx
+++ b/space-battleship/config_excel/crew_config.xlsx
@@ -1251,7 +1251,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1461,6 +1461,46 @@
         <v>25</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>hyperspace_duration_k</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>船员等级越高，异空间挂机耗时越短。</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>hyperspace_luck_per_level</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>每级增加幸运；探索奖励的词缀品阶可额外重抽并保留最好结果。</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Integrate tutorial and no-ticket hyperspace review candidate
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/crew_config.xlsx
+++ b/space-battleship/config_excel/crew_config.xlsx
@@ -1251,7 +1251,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1461,6 +1461,46 @@
         <v>25</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>hyperspace_duration_k</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>船员等级越高，异空间挂机耗时越短。</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>hyperspace_luck_per_level</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>每级增加幸运；探索奖励的词缀品阶可额外重抽并保留最好结果。</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Integrate reviewed tutorial and hyperspace changes for user playtest
Runtime code and assets match reviewed candidate 9075451. Preserve existing main evidence trees; exclude new reports, screenshots, saves and caches. Per user request, publish for local playtest while overall performance remains unresolved. DPS presentation work is not included. Flat ship compositor remains opt-in.
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/crew_config.xlsx
+++ b/space-battleship/config_excel/crew_config.xlsx
@@ -1251,7 +1251,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1461,6 +1461,46 @@
         <v>25</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>hyperspace_duration_k</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>船员等级越高，异空间挂机耗时越短。</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>hyperspace_luck_per_level</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>每级增加幸运；探索奖励的词缀品阶可额外重抽并保留最好结果。</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>